<commit_message>
test: add complete selenium appium e2e and performance testing
</commit_message>
<xml_diff>
--- a/reports/selenium/TablePulse_Web_Selenium_Test_Report.xlsx
+++ b/reports/selenium/TablePulse_Web_Selenium_Test_Report.xlsx
@@ -412,7 +412,7 @@
         <v>Generated Date</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-02T17:53:56.927Z</v>
+        <v>2026-10-05T12:50:50.344Z</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>Total Execution Duration</v>
       </c>
       <c r="B15" t="str">
-        <v>361.34 seconds</v>
+        <v>348.08 seconds</v>
       </c>
       <c r="C15" t="str">
         <v/>
@@ -641,7 +641,7 @@
         <v>Critical</v>
       </c>
       <c r="M2">
-        <v>693</v>
+        <v>738</v>
       </c>
       <c r="N2" t="str">
         <v>N/A</v>
@@ -693,7 +693,7 @@
         <v>Critical</v>
       </c>
       <c r="M3">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="N3" t="str">
         <v>N/A</v>
@@ -745,7 +745,7 @@
         <v>Critical</v>
       </c>
       <c r="M4">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="N4" t="str">
         <v>N/A</v>
@@ -797,7 +797,7 @@
         <v>Critical</v>
       </c>
       <c r="M5">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="N5" t="str">
         <v>N/A</v>
@@ -849,7 +849,7 @@
         <v>Critical</v>
       </c>
       <c r="M6">
-        <v>145</v>
+        <v>173</v>
       </c>
       <c r="N6" t="str">
         <v>N/A</v>
@@ -901,7 +901,7 @@
         <v>Critical</v>
       </c>
       <c r="M7">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="N7" t="str">
         <v>N/A</v>
@@ -953,7 +953,7 @@
         <v>Critical</v>
       </c>
       <c r="M8">
-        <v>139</v>
+        <v>166</v>
       </c>
       <c r="N8" t="str">
         <v>N/A</v>
@@ -1005,7 +1005,7 @@
         <v>Critical</v>
       </c>
       <c r="M9">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="N9" t="str">
         <v>N/A</v>
@@ -1057,7 +1057,7 @@
         <v>Critical</v>
       </c>
       <c r="M10">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N10" t="str">
         <v>N/A</v>
@@ -1109,7 +1109,7 @@
         <v>Critical</v>
       </c>
       <c r="M11">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="N11" t="str">
         <v>N/A</v>
@@ -1161,7 +1161,7 @@
         <v>Critical</v>
       </c>
       <c r="M12">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="N12" t="str">
         <v>N/A</v>
@@ -1213,7 +1213,7 @@
         <v>Critical</v>
       </c>
       <c r="M13">
-        <v>154</v>
+        <v>186</v>
       </c>
       <c r="N13" t="str">
         <v>N/A</v>
@@ -1265,7 +1265,7 @@
         <v>Critical</v>
       </c>
       <c r="M14">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N14" t="str">
         <v>N/A</v>
@@ -1317,7 +1317,7 @@
         <v>Critical</v>
       </c>
       <c r="M15">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N15" t="str">
         <v>N/A</v>
@@ -1369,7 +1369,7 @@
         <v>Critical</v>
       </c>
       <c r="M16">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="N16" t="str">
         <v>N/A</v>
@@ -1421,7 +1421,7 @@
         <v>Critical</v>
       </c>
       <c r="M17">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="N17" t="str">
         <v>N/A</v>
@@ -1473,7 +1473,7 @@
         <v>Critical</v>
       </c>
       <c r="M18">
-        <v>202</v>
+        <v>173</v>
       </c>
       <c r="N18" t="str">
         <v>N/A</v>
@@ -1525,7 +1525,7 @@
         <v>Critical</v>
       </c>
       <c r="M19">
-        <v>168</v>
+        <v>202</v>
       </c>
       <c r="N19" t="str">
         <v>N/A</v>
@@ -1577,7 +1577,7 @@
         <v>Critical</v>
       </c>
       <c r="M20">
-        <v>159</v>
+        <v>201</v>
       </c>
       <c r="N20" t="str">
         <v>N/A</v>
@@ -1629,7 +1629,7 @@
         <v>Critical</v>
       </c>
       <c r="M21">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="N21" t="str">
         <v>N/A</v>
@@ -1681,7 +1681,7 @@
         <v>Major</v>
       </c>
       <c r="M22">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="N22" t="str">
         <v>N/A</v>
@@ -1733,7 +1733,7 @@
         <v>Major</v>
       </c>
       <c r="M23">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="N23" t="str">
         <v>N/A</v>
@@ -1785,7 +1785,7 @@
         <v>Major</v>
       </c>
       <c r="M24">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="N24" t="str">
         <v>N/A</v>
@@ -1837,7 +1837,7 @@
         <v>Major</v>
       </c>
       <c r="M25">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="N25" t="str">
         <v>N/A</v>
@@ -1889,7 +1889,7 @@
         <v>Major</v>
       </c>
       <c r="M26">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="N26" t="str">
         <v>N/A</v>
@@ -1941,7 +1941,7 @@
         <v>Major</v>
       </c>
       <c r="M27">
-        <v>148</v>
+        <v>176</v>
       </c>
       <c r="N27" t="str">
         <v>N/A</v>
@@ -1993,7 +1993,7 @@
         <v>Major</v>
       </c>
       <c r="M28">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="N28" t="str">
         <v>N/A</v>
@@ -2045,7 +2045,7 @@
         <v>Major</v>
       </c>
       <c r="M29">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="N29" t="str">
         <v>N/A</v>
@@ -2097,7 +2097,7 @@
         <v>Major</v>
       </c>
       <c r="M30">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="N30" t="str">
         <v>N/A</v>
@@ -2149,7 +2149,7 @@
         <v>Major</v>
       </c>
       <c r="M31">
-        <v>190</v>
+        <v>169</v>
       </c>
       <c r="N31" t="str">
         <v>N/A</v>
@@ -2201,7 +2201,7 @@
         <v>Major</v>
       </c>
       <c r="M32">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="N32" t="str">
         <v>N/A</v>
@@ -2253,7 +2253,7 @@
         <v>Major</v>
       </c>
       <c r="M33">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="N33" t="str">
         <v>N/A</v>
@@ -2305,7 +2305,7 @@
         <v>Major</v>
       </c>
       <c r="M34">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="N34" t="str">
         <v>N/A</v>
@@ -2357,7 +2357,7 @@
         <v>Major</v>
       </c>
       <c r="M35">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="N35" t="str">
         <v>N/A</v>
@@ -2409,7 +2409,7 @@
         <v>Major</v>
       </c>
       <c r="M36">
-        <v>170</v>
+        <v>237</v>
       </c>
       <c r="N36" t="str">
         <v>N/A</v>
@@ -2461,7 +2461,7 @@
         <v>Major</v>
       </c>
       <c r="M37">
-        <v>162</v>
+        <v>190</v>
       </c>
       <c r="N37" t="str">
         <v>N/A</v>
@@ -2513,7 +2513,7 @@
         <v>Major</v>
       </c>
       <c r="M38">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="N38" t="str">
         <v>N/A</v>
@@ -2565,7 +2565,7 @@
         <v>Major</v>
       </c>
       <c r="M39">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="N39" t="str">
         <v>N/A</v>
@@ -2617,7 +2617,7 @@
         <v>Major</v>
       </c>
       <c r="M40">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="N40" t="str">
         <v>N/A</v>
@@ -2669,7 +2669,7 @@
         <v>Major</v>
       </c>
       <c r="M41">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="N41" t="str">
         <v>N/A</v>
@@ -2721,7 +2721,7 @@
         <v>Critical</v>
       </c>
       <c r="M42">
-        <v>2085</v>
+        <v>1992</v>
       </c>
       <c r="N42" t="str">
         <v>N/A</v>
@@ -2773,7 +2773,7 @@
         <v>Critical</v>
       </c>
       <c r="M43">
-        <v>2016</v>
+        <v>2010</v>
       </c>
       <c r="N43" t="str">
         <v>N/A</v>
@@ -2825,7 +2825,7 @@
         <v>Critical</v>
       </c>
       <c r="M44">
-        <v>2016</v>
+        <v>1986</v>
       </c>
       <c r="N44" t="str">
         <v>N/A</v>
@@ -2877,7 +2877,7 @@
         <v>Critical</v>
       </c>
       <c r="M45">
-        <v>2015</v>
+        <v>1998</v>
       </c>
       <c r="N45" t="str">
         <v>N/A</v>
@@ -2929,7 +2929,7 @@
         <v>Critical</v>
       </c>
       <c r="M46">
-        <v>2010</v>
+        <v>2027</v>
       </c>
       <c r="N46" t="str">
         <v>N/A</v>
@@ -2981,7 +2981,7 @@
         <v>Critical</v>
       </c>
       <c r="M47">
-        <v>2008</v>
+        <v>1981</v>
       </c>
       <c r="N47" t="str">
         <v>N/A</v>
@@ -3033,7 +3033,7 @@
         <v>Critical</v>
       </c>
       <c r="M48">
-        <v>2013</v>
+        <v>1964</v>
       </c>
       <c r="N48" t="str">
         <v>N/A</v>
@@ -3085,7 +3085,7 @@
         <v>Critical</v>
       </c>
       <c r="M49">
-        <v>2041</v>
+        <v>2033</v>
       </c>
       <c r="N49" t="str">
         <v>N/A</v>
@@ -3137,7 +3137,7 @@
         <v>Critical</v>
       </c>
       <c r="M50">
-        <v>2006</v>
+        <v>2043</v>
       </c>
       <c r="N50" t="str">
         <v>N/A</v>
@@ -3189,7 +3189,7 @@
         <v>Critical</v>
       </c>
       <c r="M51">
-        <v>2006</v>
+        <v>2019</v>
       </c>
       <c r="N51" t="str">
         <v>N/A</v>
@@ -3241,7 +3241,7 @@
         <v>Critical</v>
       </c>
       <c r="M52">
-        <v>2030</v>
+        <v>2145</v>
       </c>
       <c r="N52" t="str">
         <v>N/A</v>
@@ -3293,7 +3293,7 @@
         <v>Critical</v>
       </c>
       <c r="M53">
-        <v>2055</v>
+        <v>2040</v>
       </c>
       <c r="N53" t="str">
         <v>N/A</v>
@@ -3345,7 +3345,7 @@
         <v>Critical</v>
       </c>
       <c r="M54">
-        <v>2042</v>
+        <v>2014</v>
       </c>
       <c r="N54" t="str">
         <v>N/A</v>
@@ -3397,7 +3397,7 @@
         <v>Critical</v>
       </c>
       <c r="M55">
-        <v>2205</v>
+        <v>2023</v>
       </c>
       <c r="N55" t="str">
         <v>N/A</v>
@@ -3449,7 +3449,7 @@
         <v>Critical</v>
       </c>
       <c r="M56">
-        <v>2045</v>
+        <v>2097</v>
       </c>
       <c r="N56" t="str">
         <v>N/A</v>
@@ -3501,7 +3501,7 @@
         <v>Critical</v>
       </c>
       <c r="M57">
-        <v>2017</v>
+        <v>1992</v>
       </c>
       <c r="N57" t="str">
         <v>N/A</v>
@@ -3553,7 +3553,7 @@
         <v>Critical</v>
       </c>
       <c r="M58">
-        <v>2198</v>
+        <v>2104</v>
       </c>
       <c r="N58" t="str">
         <v>N/A</v>
@@ -3605,7 +3605,7 @@
         <v>Critical</v>
       </c>
       <c r="M59">
-        <v>2004</v>
+        <v>1988</v>
       </c>
       <c r="N59" t="str">
         <v>N/A</v>
@@ -3657,7 +3657,7 @@
         <v>Critical</v>
       </c>
       <c r="M60">
-        <v>2055</v>
+        <v>2069</v>
       </c>
       <c r="N60" t="str">
         <v>N/A</v>
@@ -3709,7 +3709,7 @@
         <v>Critical</v>
       </c>
       <c r="M61">
-        <v>2083</v>
+        <v>1968</v>
       </c>
       <c r="N61" t="str">
         <v>N/A</v>
@@ -3761,7 +3761,7 @@
         <v>Critical</v>
       </c>
       <c r="M62">
-        <v>2027</v>
+        <v>2140</v>
       </c>
       <c r="N62" t="str">
         <v>N/A</v>
@@ -3813,7 +3813,7 @@
         <v>Critical</v>
       </c>
       <c r="M63">
-        <v>2019</v>
+        <v>2035</v>
       </c>
       <c r="N63" t="str">
         <v>N/A</v>
@@ -3865,7 +3865,7 @@
         <v>Critical</v>
       </c>
       <c r="M64">
-        <v>2010</v>
+        <v>2114</v>
       </c>
       <c r="N64" t="str">
         <v>N/A</v>
@@ -3917,7 +3917,7 @@
         <v>Critical</v>
       </c>
       <c r="M65">
-        <v>2037</v>
+        <v>2148</v>
       </c>
       <c r="N65" t="str">
         <v>N/A</v>
@@ -3969,7 +3969,7 @@
         <v>Critical</v>
       </c>
       <c r="M66">
-        <v>2008</v>
+        <v>2106</v>
       </c>
       <c r="N66" t="str">
         <v>N/A</v>
@@ -4021,7 +4021,7 @@
         <v>Major</v>
       </c>
       <c r="M67">
-        <v>1172</v>
+        <v>449</v>
       </c>
       <c r="N67" t="str">
         <v>N/A</v>
@@ -4073,7 +4073,7 @@
         <v>Major</v>
       </c>
       <c r="M68">
-        <v>1198</v>
+        <v>489</v>
       </c>
       <c r="N68" t="str">
         <v>N/A</v>
@@ -4125,7 +4125,7 @@
         <v>Major</v>
       </c>
       <c r="M69">
-        <v>1181</v>
+        <v>405</v>
       </c>
       <c r="N69" t="str">
         <v>N/A</v>
@@ -4177,7 +4177,7 @@
         <v>Major</v>
       </c>
       <c r="M70">
-        <v>1176</v>
+        <v>379</v>
       </c>
       <c r="N70" t="str">
         <v>N/A</v>
@@ -4229,7 +4229,7 @@
         <v>Major</v>
       </c>
       <c r="M71">
-        <v>1202</v>
+        <v>345</v>
       </c>
       <c r="N71" t="str">
         <v>N/A</v>
@@ -4281,7 +4281,7 @@
         <v>Major</v>
       </c>
       <c r="M72">
-        <v>1189</v>
+        <v>376</v>
       </c>
       <c r="N72" t="str">
         <v>N/A</v>
@@ -4333,7 +4333,7 @@
         <v>Major</v>
       </c>
       <c r="M73">
-        <v>1159</v>
+        <v>378</v>
       </c>
       <c r="N73" t="str">
         <v>N/A</v>
@@ -4385,7 +4385,7 @@
         <v>Major</v>
       </c>
       <c r="M74">
-        <v>1173</v>
+        <v>355</v>
       </c>
       <c r="N74" t="str">
         <v>N/A</v>
@@ -4437,7 +4437,7 @@
         <v>Major</v>
       </c>
       <c r="M75">
-        <v>1181</v>
+        <v>360</v>
       </c>
       <c r="N75" t="str">
         <v>N/A</v>
@@ -4489,7 +4489,7 @@
         <v>Major</v>
       </c>
       <c r="M76">
-        <v>1201</v>
+        <v>372</v>
       </c>
       <c r="N76" t="str">
         <v>N/A</v>
@@ -4541,7 +4541,7 @@
         <v>Major</v>
       </c>
       <c r="M77">
-        <v>1191</v>
+        <v>407</v>
       </c>
       <c r="N77" t="str">
         <v>N/A</v>
@@ -4593,7 +4593,7 @@
         <v>Major</v>
       </c>
       <c r="M78">
-        <v>1160</v>
+        <v>436</v>
       </c>
       <c r="N78" t="str">
         <v>N/A</v>
@@ -4645,7 +4645,7 @@
         <v>Major</v>
       </c>
       <c r="M79">
-        <v>1197</v>
+        <v>346</v>
       </c>
       <c r="N79" t="str">
         <v>N/A</v>
@@ -4697,7 +4697,7 @@
         <v>Major</v>
       </c>
       <c r="M80">
-        <v>1203</v>
+        <v>433</v>
       </c>
       <c r="N80" t="str">
         <v>N/A</v>
@@ -4749,7 +4749,7 @@
         <v>Major</v>
       </c>
       <c r="M81">
-        <v>1171</v>
+        <v>399</v>
       </c>
       <c r="N81" t="str">
         <v>N/A</v>
@@ -4801,7 +4801,7 @@
         <v>Major</v>
       </c>
       <c r="M82">
-        <v>1188</v>
+        <v>373</v>
       </c>
       <c r="N82" t="str">
         <v>N/A</v>
@@ -4853,7 +4853,7 @@
         <v>Major</v>
       </c>
       <c r="M83">
-        <v>1176</v>
+        <v>374</v>
       </c>
       <c r="N83" t="str">
         <v>N/A</v>
@@ -4905,7 +4905,7 @@
         <v>Major</v>
       </c>
       <c r="M84">
-        <v>1176</v>
+        <v>402</v>
       </c>
       <c r="N84" t="str">
         <v>N/A</v>
@@ -4957,7 +4957,7 @@
         <v>Major</v>
       </c>
       <c r="M85">
-        <v>1207</v>
+        <v>362</v>
       </c>
       <c r="N85" t="str">
         <v>N/A</v>
@@ -5009,7 +5009,7 @@
         <v>Major</v>
       </c>
       <c r="M86">
-        <v>1189</v>
+        <v>372</v>
       </c>
       <c r="N86" t="str">
         <v>N/A</v>
@@ -5061,7 +5061,7 @@
         <v>Critical</v>
       </c>
       <c r="M87">
-        <v>1678</v>
+        <v>1727</v>
       </c>
       <c r="N87" t="str">
         <v>N/A</v>
@@ -5113,7 +5113,7 @@
         <v>Critical</v>
       </c>
       <c r="M88">
-        <v>1679</v>
+        <v>1715</v>
       </c>
       <c r="N88" t="str">
         <v>N/A</v>
@@ -5165,7 +5165,7 @@
         <v>Critical</v>
       </c>
       <c r="M89">
-        <v>1671</v>
+        <v>1705</v>
       </c>
       <c r="N89" t="str">
         <v>N/A</v>
@@ -5217,7 +5217,7 @@
         <v>Critical</v>
       </c>
       <c r="M90">
-        <v>1698</v>
+        <v>1690</v>
       </c>
       <c r="N90" t="str">
         <v>N/A</v>
@@ -5269,7 +5269,7 @@
         <v>Critical</v>
       </c>
       <c r="M91">
-        <v>1705</v>
+        <v>1746</v>
       </c>
       <c r="N91" t="str">
         <v>N/A</v>
@@ -5321,7 +5321,7 @@
         <v>Critical</v>
       </c>
       <c r="M92">
-        <v>1715</v>
+        <v>1750</v>
       </c>
       <c r="N92" t="str">
         <v>N/A</v>
@@ -5373,7 +5373,7 @@
         <v>Critical</v>
       </c>
       <c r="M93">
-        <v>1678</v>
+        <v>1799</v>
       </c>
       <c r="N93" t="str">
         <v>N/A</v>
@@ -5425,7 +5425,7 @@
         <v>Critical</v>
       </c>
       <c r="M94">
-        <v>1688</v>
+        <v>1776</v>
       </c>
       <c r="N94" t="str">
         <v>N/A</v>
@@ -5477,7 +5477,7 @@
         <v>Critical</v>
       </c>
       <c r="M95">
-        <v>1671</v>
+        <v>1733</v>
       </c>
       <c r="N95" t="str">
         <v>N/A</v>
@@ -5529,7 +5529,7 @@
         <v>Critical</v>
       </c>
       <c r="M96">
-        <v>1675</v>
+        <v>1723</v>
       </c>
       <c r="N96" t="str">
         <v>N/A</v>
@@ -5581,7 +5581,7 @@
         <v>Critical</v>
       </c>
       <c r="M97">
-        <v>1702</v>
+        <v>1774</v>
       </c>
       <c r="N97" t="str">
         <v>N/A</v>
@@ -5633,7 +5633,7 @@
         <v>Critical</v>
       </c>
       <c r="M98">
-        <v>1685</v>
+        <v>1795</v>
       </c>
       <c r="N98" t="str">
         <v>N/A</v>
@@ -5685,7 +5685,7 @@
         <v>Critical</v>
       </c>
       <c r="M99">
-        <v>1711</v>
+        <v>1769</v>
       </c>
       <c r="N99" t="str">
         <v>N/A</v>
@@ -5737,7 +5737,7 @@
         <v>Critical</v>
       </c>
       <c r="M100">
-        <v>1713</v>
+        <v>1717</v>
       </c>
       <c r="N100" t="str">
         <v>N/A</v>
@@ -5789,7 +5789,7 @@
         <v>Critical</v>
       </c>
       <c r="M101">
-        <v>1678</v>
+        <v>1786</v>
       </c>
       <c r="N101" t="str">
         <v>N/A</v>
@@ -5841,7 +5841,7 @@
         <v>Critical</v>
       </c>
       <c r="M102">
-        <v>1686</v>
+        <v>1779</v>
       </c>
       <c r="N102" t="str">
         <v>N/A</v>
@@ -5893,7 +5893,7 @@
         <v>Critical</v>
       </c>
       <c r="M103">
-        <v>1672</v>
+        <v>1702</v>
       </c>
       <c r="N103" t="str">
         <v>N/A</v>
@@ -5945,7 +5945,7 @@
         <v>Critical</v>
       </c>
       <c r="M104">
-        <v>1727</v>
+        <v>1691</v>
       </c>
       <c r="N104" t="str">
         <v>N/A</v>
@@ -5997,7 +5997,7 @@
         <v>Critical</v>
       </c>
       <c r="M105">
-        <v>1707</v>
+        <v>1693</v>
       </c>
       <c r="N105" t="str">
         <v>N/A</v>
@@ -6049,7 +6049,7 @@
         <v>Critical</v>
       </c>
       <c r="M106">
-        <v>1706</v>
+        <v>1741</v>
       </c>
       <c r="N106" t="str">
         <v>N/A</v>
@@ -6101,7 +6101,7 @@
         <v>Critical</v>
       </c>
       <c r="M107">
-        <v>1678</v>
+        <v>1761</v>
       </c>
       <c r="N107" t="str">
         <v>N/A</v>
@@ -6153,7 +6153,7 @@
         <v>Critical</v>
       </c>
       <c r="M108">
-        <v>1666</v>
+        <v>1703</v>
       </c>
       <c r="N108" t="str">
         <v>N/A</v>
@@ -6205,7 +6205,7 @@
         <v>Critical</v>
       </c>
       <c r="M109">
-        <v>1676</v>
+        <v>1706</v>
       </c>
       <c r="N109" t="str">
         <v>N/A</v>
@@ -6257,7 +6257,7 @@
         <v>Critical</v>
       </c>
       <c r="M110">
-        <v>1753</v>
+        <v>1718</v>
       </c>
       <c r="N110" t="str">
         <v>N/A</v>
@@ -6309,7 +6309,7 @@
         <v>Critical</v>
       </c>
       <c r="M111">
-        <v>1686</v>
+        <v>1768</v>
       </c>
       <c r="N111" t="str">
         <v>N/A</v>
@@ -6361,7 +6361,7 @@
         <v>Major</v>
       </c>
       <c r="M112">
-        <v>2373</v>
+        <v>2368</v>
       </c>
       <c r="N112" t="str">
         <v>N/A</v>
@@ -6413,7 +6413,7 @@
         <v>Major</v>
       </c>
       <c r="M113">
-        <v>2364</v>
+        <v>2391</v>
       </c>
       <c r="N113" t="str">
         <v>N/A</v>
@@ -6465,7 +6465,7 @@
         <v>Major</v>
       </c>
       <c r="M114">
-        <v>2334</v>
+        <v>2406</v>
       </c>
       <c r="N114" t="str">
         <v>N/A</v>
@@ -6517,7 +6517,7 @@
         <v>Major</v>
       </c>
       <c r="M115">
-        <v>2330</v>
+        <v>2323</v>
       </c>
       <c r="N115" t="str">
         <v>N/A</v>
@@ -6569,7 +6569,7 @@
         <v>Major</v>
       </c>
       <c r="M116">
-        <v>2312</v>
+        <v>2404</v>
       </c>
       <c r="N116" t="str">
         <v>N/A</v>
@@ -6621,7 +6621,7 @@
         <v>Major</v>
       </c>
       <c r="M117">
-        <v>2295</v>
+        <v>2363</v>
       </c>
       <c r="N117" t="str">
         <v>N/A</v>
@@ -6673,7 +6673,7 @@
         <v>Major</v>
       </c>
       <c r="M118">
-        <v>2290</v>
+        <v>2358</v>
       </c>
       <c r="N118" t="str">
         <v>N/A</v>
@@ -6725,7 +6725,7 @@
         <v>Major</v>
       </c>
       <c r="M119">
-        <v>2323</v>
+        <v>2305</v>
       </c>
       <c r="N119" t="str">
         <v>N/A</v>
@@ -6777,7 +6777,7 @@
         <v>Major</v>
       </c>
       <c r="M120">
-        <v>2353</v>
+        <v>2394</v>
       </c>
       <c r="N120" t="str">
         <v>N/A</v>
@@ -6829,7 +6829,7 @@
         <v>Major</v>
       </c>
       <c r="M121">
-        <v>2386</v>
+        <v>2312</v>
       </c>
       <c r="N121" t="str">
         <v>N/A</v>
@@ -6881,7 +6881,7 @@
         <v>Major</v>
       </c>
       <c r="M122">
-        <v>2310</v>
+        <v>2304</v>
       </c>
       <c r="N122" t="str">
         <v>N/A</v>
@@ -6933,7 +6933,7 @@
         <v>Major</v>
       </c>
       <c r="M123">
-        <v>2347</v>
+        <v>2297</v>
       </c>
       <c r="N123" t="str">
         <v>N/A</v>
@@ -6985,7 +6985,7 @@
         <v>Major</v>
       </c>
       <c r="M124">
-        <v>2332</v>
+        <v>2321</v>
       </c>
       <c r="N124" t="str">
         <v>N/A</v>
@@ -7037,7 +7037,7 @@
         <v>Major</v>
       </c>
       <c r="M125">
-        <v>2301</v>
+        <v>2342</v>
       </c>
       <c r="N125" t="str">
         <v>N/A</v>
@@ -7089,7 +7089,7 @@
         <v>Major</v>
       </c>
       <c r="M126">
-        <v>2352</v>
+        <v>2339</v>
       </c>
       <c r="N126" t="str">
         <v>N/A</v>
@@ -7141,7 +7141,7 @@
         <v>Major</v>
       </c>
       <c r="M127">
-        <v>2338</v>
+        <v>2288</v>
       </c>
       <c r="N127" t="str">
         <v>N/A</v>
@@ -7193,7 +7193,7 @@
         <v>Major</v>
       </c>
       <c r="M128">
-        <v>2344</v>
+        <v>2324</v>
       </c>
       <c r="N128" t="str">
         <v>N/A</v>
@@ -7245,7 +7245,7 @@
         <v>Major</v>
       </c>
       <c r="M129">
-        <v>2312</v>
+        <v>2349</v>
       </c>
       <c r="N129" t="str">
         <v>N/A</v>
@@ -7297,7 +7297,7 @@
         <v>Major</v>
       </c>
       <c r="M130">
-        <v>2304</v>
+        <v>2408</v>
       </c>
       <c r="N130" t="str">
         <v>N/A</v>
@@ -7349,7 +7349,7 @@
         <v>Major</v>
       </c>
       <c r="M131">
-        <v>2432</v>
+        <v>2339</v>
       </c>
       <c r="N131" t="str">
         <v>N/A</v>
@@ -7401,7 +7401,7 @@
         <v>Major</v>
       </c>
       <c r="M132">
-        <v>2336</v>
+        <v>2340</v>
       </c>
       <c r="N132" t="str">
         <v>N/A</v>
@@ -7453,7 +7453,7 @@
         <v>Major</v>
       </c>
       <c r="M133">
-        <v>2326</v>
+        <v>2411</v>
       </c>
       <c r="N133" t="str">
         <v>N/A</v>
@@ -7505,7 +7505,7 @@
         <v>Major</v>
       </c>
       <c r="M134">
-        <v>2308</v>
+        <v>2310</v>
       </c>
       <c r="N134" t="str">
         <v>N/A</v>
@@ -7557,7 +7557,7 @@
         <v>Major</v>
       </c>
       <c r="M135">
-        <v>2299</v>
+        <v>2333</v>
       </c>
       <c r="N135" t="str">
         <v>N/A</v>
@@ -7609,7 +7609,7 @@
         <v>Major</v>
       </c>
       <c r="M136">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="N136" t="str">
         <v>N/A</v>
@@ -7661,7 +7661,7 @@
         <v>Critical</v>
       </c>
       <c r="M137">
-        <v>1707</v>
+        <v>1737</v>
       </c>
       <c r="N137" t="str">
         <v>N/A</v>
@@ -7765,7 +7765,7 @@
         <v>Critical</v>
       </c>
       <c r="M139">
-        <v>1691</v>
+        <v>1714</v>
       </c>
       <c r="N139" t="str">
         <v>N/A</v>
@@ -7817,7 +7817,7 @@
         <v>Critical</v>
       </c>
       <c r="M140">
-        <v>1681</v>
+        <v>1730</v>
       </c>
       <c r="N140" t="str">
         <v>N/A</v>
@@ -7869,7 +7869,7 @@
         <v>Critical</v>
       </c>
       <c r="M141">
-        <v>1676</v>
+        <v>1692</v>
       </c>
       <c r="N141" t="str">
         <v>N/A</v>
@@ -7921,7 +7921,7 @@
         <v>Critical</v>
       </c>
       <c r="M142">
-        <v>1681</v>
+        <v>1690</v>
       </c>
       <c r="N142" t="str">
         <v>N/A</v>
@@ -7973,7 +7973,7 @@
         <v>Critical</v>
       </c>
       <c r="M143">
-        <v>1711</v>
+        <v>1690</v>
       </c>
       <c r="N143" t="str">
         <v>N/A</v>
@@ -8025,7 +8025,7 @@
         <v>Critical</v>
       </c>
       <c r="M144">
-        <v>1691</v>
+        <v>1724</v>
       </c>
       <c r="N144" t="str">
         <v>N/A</v>
@@ -8077,7 +8077,7 @@
         <v>Critical</v>
       </c>
       <c r="M145">
-        <v>1686</v>
+        <v>1745</v>
       </c>
       <c r="N145" t="str">
         <v>N/A</v>
@@ -8129,7 +8129,7 @@
         <v>Critical</v>
       </c>
       <c r="M146">
-        <v>1681</v>
+        <v>1720</v>
       </c>
       <c r="N146" t="str">
         <v>N/A</v>
@@ -8181,7 +8181,7 @@
         <v>Critical</v>
       </c>
       <c r="M147">
-        <v>1664</v>
+        <v>1701</v>
       </c>
       <c r="N147" t="str">
         <v>N/A</v>
@@ -8233,7 +8233,7 @@
         <v>Critical</v>
       </c>
       <c r="M148">
-        <v>1699</v>
+        <v>1685</v>
       </c>
       <c r="N148" t="str">
         <v>N/A</v>
@@ -8285,7 +8285,7 @@
         <v>Critical</v>
       </c>
       <c r="M149">
-        <v>1693</v>
+        <v>1712</v>
       </c>
       <c r="N149" t="str">
         <v>N/A</v>
@@ -8337,7 +8337,7 @@
         <v>Critical</v>
       </c>
       <c r="M150">
-        <v>1715</v>
+        <v>1729</v>
       </c>
       <c r="N150" t="str">
         <v>N/A</v>
@@ -8389,7 +8389,7 @@
         <v>Critical</v>
       </c>
       <c r="M151">
-        <v>1676</v>
+        <v>1736</v>
       </c>
       <c r="N151" t="str">
         <v>N/A</v>
@@ -8441,7 +8441,7 @@
         <v>Critical</v>
       </c>
       <c r="M152">
-        <v>1703</v>
+        <v>1711</v>
       </c>
       <c r="N152" t="str">
         <v>N/A</v>
@@ -8493,7 +8493,7 @@
         <v>Critical</v>
       </c>
       <c r="M153">
-        <v>1700</v>
+        <v>1687</v>
       </c>
       <c r="N153" t="str">
         <v>N/A</v>
@@ -8545,7 +8545,7 @@
         <v>Critical</v>
       </c>
       <c r="M154">
-        <v>1695</v>
+        <v>1683</v>
       </c>
       <c r="N154" t="str">
         <v>N/A</v>
@@ -8597,7 +8597,7 @@
         <v>Critical</v>
       </c>
       <c r="M155">
-        <v>1699</v>
+        <v>1714</v>
       </c>
       <c r="N155" t="str">
         <v>N/A</v>
@@ -8649,7 +8649,7 @@
         <v>Critical</v>
       </c>
       <c r="M156">
-        <v>1733</v>
+        <v>1725</v>
       </c>
       <c r="N156" t="str">
         <v>N/A</v>
@@ -8701,7 +8701,7 @@
         <v>Critical</v>
       </c>
       <c r="M157">
-        <v>1687</v>
+        <v>1701</v>
       </c>
       <c r="N157" t="str">
         <v>N/A</v>
@@ -8753,7 +8753,7 @@
         <v>Critical</v>
       </c>
       <c r="M158">
-        <v>1698</v>
+        <v>1714</v>
       </c>
       <c r="N158" t="str">
         <v>N/A</v>
@@ -8805,7 +8805,7 @@
         <v>Critical</v>
       </c>
       <c r="M159">
-        <v>1697</v>
+        <v>1715</v>
       </c>
       <c r="N159" t="str">
         <v>N/A</v>
@@ -8857,7 +8857,7 @@
         <v>Critical</v>
       </c>
       <c r="M160">
-        <v>1682</v>
+        <v>1698</v>
       </c>
       <c r="N160" t="str">
         <v>N/A</v>
@@ -8909,7 +8909,7 @@
         <v>Critical</v>
       </c>
       <c r="M161">
-        <v>1671</v>
+        <v>1709</v>
       </c>
       <c r="N161" t="str">
         <v>N/A</v>
@@ -8961,7 +8961,7 @@
         <v>Critical</v>
       </c>
       <c r="M162">
-        <v>1695</v>
+        <v>1739</v>
       </c>
       <c r="N162" t="str">
         <v>N/A</v>
@@ -9013,7 +9013,7 @@
         <v>Critical</v>
       </c>
       <c r="M163">
-        <v>1686</v>
+        <v>1702</v>
       </c>
       <c r="N163" t="str">
         <v>N/A</v>
@@ -9065,7 +9065,7 @@
         <v>Critical</v>
       </c>
       <c r="M164">
-        <v>1712</v>
+        <v>1685</v>
       </c>
       <c r="N164" t="str">
         <v>N/A</v>
@@ -9117,7 +9117,7 @@
         <v>Critical</v>
       </c>
       <c r="M165">
-        <v>1688</v>
+        <v>1766</v>
       </c>
       <c r="N165" t="str">
         <v>N/A</v>
@@ -9169,7 +9169,7 @@
         <v>Critical</v>
       </c>
       <c r="M166">
-        <v>1697</v>
+        <v>1756</v>
       </c>
       <c r="N166" t="str">
         <v>N/A</v>
@@ -9221,7 +9221,7 @@
         <v>Critical</v>
       </c>
       <c r="M167">
-        <v>1680</v>
+        <v>1701</v>
       </c>
       <c r="N167" t="str">
         <v>N/A</v>
@@ -9273,7 +9273,7 @@
         <v>Critical</v>
       </c>
       <c r="M168">
-        <v>1680</v>
+        <v>1696</v>
       </c>
       <c r="N168" t="str">
         <v>N/A</v>
@@ -9325,7 +9325,7 @@
         <v>Critical</v>
       </c>
       <c r="M169">
-        <v>1694</v>
+        <v>1700</v>
       </c>
       <c r="N169" t="str">
         <v>N/A</v>
@@ -9377,7 +9377,7 @@
         <v>Critical</v>
       </c>
       <c r="M170">
-        <v>1683</v>
+        <v>1716</v>
       </c>
       <c r="N170" t="str">
         <v>N/A</v>
@@ -9429,7 +9429,7 @@
         <v>Critical</v>
       </c>
       <c r="M171">
-        <v>1679</v>
+        <v>1723</v>
       </c>
       <c r="N171" t="str">
         <v>N/A</v>
@@ -9481,7 +9481,7 @@
         <v>Critical</v>
       </c>
       <c r="M172">
-        <v>1669</v>
+        <v>1720</v>
       </c>
       <c r="N172" t="str">
         <v>N/A</v>
@@ -9533,7 +9533,7 @@
         <v>Critical</v>
       </c>
       <c r="M173">
-        <v>1677</v>
+        <v>1703</v>
       </c>
       <c r="N173" t="str">
         <v>N/A</v>
@@ -9585,7 +9585,7 @@
         <v>Critical</v>
       </c>
       <c r="M174">
-        <v>1690</v>
+        <v>1731</v>
       </c>
       <c r="N174" t="str">
         <v>N/A</v>
@@ -9637,7 +9637,7 @@
         <v>Critical</v>
       </c>
       <c r="M175">
-        <v>1675</v>
+        <v>1682</v>
       </c>
       <c r="N175" t="str">
         <v>N/A</v>
@@ -9689,7 +9689,7 @@
         <v>Critical</v>
       </c>
       <c r="M176">
-        <v>1705</v>
+        <v>1701</v>
       </c>
       <c r="N176" t="str">
         <v>N/A</v>
@@ -9741,7 +9741,7 @@
         <v>Critical</v>
       </c>
       <c r="M177">
-        <v>1666</v>
+        <v>1734</v>
       </c>
       <c r="N177" t="str">
         <v>N/A</v>
@@ -9793,7 +9793,7 @@
         <v>Critical</v>
       </c>
       <c r="M178">
-        <v>1696</v>
+        <v>1721</v>
       </c>
       <c r="N178" t="str">
         <v>N/A</v>
@@ -9845,7 +9845,7 @@
         <v>Critical</v>
       </c>
       <c r="M179">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="N179" t="str">
         <v>N/A</v>
@@ -9897,7 +9897,7 @@
         <v>Critical</v>
       </c>
       <c r="M180">
-        <v>1669</v>
+        <v>1687</v>
       </c>
       <c r="N180" t="str">
         <v>N/A</v>
@@ -9949,7 +9949,7 @@
         <v>Critical</v>
       </c>
       <c r="M181">
-        <v>1672</v>
+        <v>1710</v>
       </c>
       <c r="N181" t="str">
         <v>N/A</v>
@@ -10000,7 +10000,7 @@
         <v>Major</v>
       </c>
       <c r="M182">
-        <v>1706</v>
+        <v>1721</v>
       </c>
       <c r="N182" t="str">
         <v>N/A</v>
@@ -10051,7 +10051,7 @@
         <v>Major</v>
       </c>
       <c r="M183">
-        <v>1673</v>
+        <v>1694</v>
       </c>
       <c r="N183" t="str">
         <v>N/A</v>
@@ -10102,7 +10102,7 @@
         <v>Major</v>
       </c>
       <c r="M184">
-        <v>1665</v>
+        <v>1673</v>
       </c>
       <c r="N184" t="str">
         <v>N/A</v>
@@ -10153,7 +10153,7 @@
         <v>Major</v>
       </c>
       <c r="M185">
-        <v>1668</v>
+        <v>1709</v>
       </c>
       <c r="N185" t="str">
         <v>N/A</v>
@@ -10204,7 +10204,7 @@
         <v>Major</v>
       </c>
       <c r="M186">
-        <v>1700</v>
+        <v>1729</v>
       </c>
       <c r="N186" t="str">
         <v>N/A</v>
@@ -10255,7 +10255,7 @@
         <v>Major</v>
       </c>
       <c r="M187">
-        <v>1660</v>
+        <v>1703</v>
       </c>
       <c r="N187" t="str">
         <v>N/A</v>
@@ -10306,7 +10306,7 @@
         <v>Major</v>
       </c>
       <c r="M188">
-        <v>1668</v>
+        <v>1706</v>
       </c>
       <c r="N188" t="str">
         <v>N/A</v>
@@ -10357,7 +10357,7 @@
         <v>Major</v>
       </c>
       <c r="M189">
-        <v>1674</v>
+        <v>1737</v>
       </c>
       <c r="N189" t="str">
         <v>N/A</v>
@@ -10408,7 +10408,7 @@
         <v>Major</v>
       </c>
       <c r="M190">
-        <v>1673</v>
+        <v>1700</v>
       </c>
       <c r="N190" t="str">
         <v>N/A</v>
@@ -10459,7 +10459,7 @@
         <v>Major</v>
       </c>
       <c r="M191">
-        <v>1669</v>
+        <v>1690</v>
       </c>
       <c r="N191" t="str">
         <v>N/A</v>
@@ -10510,7 +10510,7 @@
         <v>Major</v>
       </c>
       <c r="M192">
-        <v>1678</v>
+        <v>1681</v>
       </c>
       <c r="N192" t="str">
         <v>N/A</v>
@@ -10561,7 +10561,7 @@
         <v>Major</v>
       </c>
       <c r="M193">
-        <v>1679</v>
+        <v>1702</v>
       </c>
       <c r="N193" t="str">
         <v>N/A</v>
@@ -10612,7 +10612,7 @@
         <v>Major</v>
       </c>
       <c r="M194">
-        <v>1685</v>
+        <v>1724</v>
       </c>
       <c r="N194" t="str">
         <v>N/A</v>
@@ -10663,7 +10663,7 @@
         <v>Major</v>
       </c>
       <c r="M195">
-        <v>1693</v>
+        <v>1711</v>
       </c>
       <c r="N195" t="str">
         <v>N/A</v>
@@ -10714,7 +10714,7 @@
         <v>Major</v>
       </c>
       <c r="M196">
-        <v>1676</v>
+        <v>1760</v>
       </c>
       <c r="N196" t="str">
         <v>N/A</v>
@@ -10765,7 +10765,7 @@
         <v>Critical</v>
       </c>
       <c r="M197">
-        <v>1788</v>
+        <v>1804</v>
       </c>
       <c r="N197" t="str">
         <v>N/A</v>
@@ -10816,7 +10816,7 @@
         <v>Critical</v>
       </c>
       <c r="M198">
-        <v>1800</v>
+        <v>1842</v>
       </c>
       <c r="N198" t="str">
         <v>N/A</v>
@@ -10867,7 +10867,7 @@
         <v>Critical</v>
       </c>
       <c r="M199">
-        <v>1859</v>
+        <v>1769</v>
       </c>
       <c r="N199" t="str">
         <v>N/A</v>
@@ -10918,7 +10918,7 @@
         <v>Critical</v>
       </c>
       <c r="M200">
-        <v>1812</v>
+        <v>1763</v>
       </c>
       <c r="N200" t="str">
         <v>N/A</v>
@@ -10969,7 +10969,7 @@
         <v>Critical</v>
       </c>
       <c r="M201">
-        <v>1778</v>
+        <v>1765</v>
       </c>
       <c r="N201" t="str">
         <v>N/A</v>
@@ -11020,7 +11020,7 @@
         <v>Critical</v>
       </c>
       <c r="M202">
-        <v>1785</v>
+        <v>1790</v>
       </c>
       <c r="N202" t="str">
         <v>N/A</v>
@@ -11071,7 +11071,7 @@
         <v>Critical</v>
       </c>
       <c r="M203">
-        <v>1780</v>
+        <v>1832</v>
       </c>
       <c r="N203" t="str">
         <v>N/A</v>
@@ -11122,7 +11122,7 @@
         <v>Critical</v>
       </c>
       <c r="M204">
-        <v>1818</v>
+        <v>1780</v>
       </c>
       <c r="N204" t="str">
         <v>N/A</v>
@@ -11173,7 +11173,7 @@
         <v>Critical</v>
       </c>
       <c r="M205">
-        <v>1772</v>
+        <v>1780</v>
       </c>
       <c r="N205" t="str">
         <v>N/A</v>
@@ -11224,7 +11224,7 @@
         <v>Critical</v>
       </c>
       <c r="M206">
-        <v>1779</v>
+        <v>1806</v>
       </c>
       <c r="N206" t="str">
         <v>N/A</v>
@@ -11275,7 +11275,7 @@
         <v>Critical</v>
       </c>
       <c r="M207">
-        <v>1747</v>
+        <v>1805</v>
       </c>
       <c r="N207" t="str">
         <v>N/A</v>
@@ -11326,7 +11326,7 @@
         <v>Critical</v>
       </c>
       <c r="M208">
-        <v>1789</v>
+        <v>1800</v>
       </c>
       <c r="N208" t="str">
         <v>N/A</v>
@@ -11377,7 +11377,7 @@
         <v>Critical</v>
       </c>
       <c r="M209">
-        <v>1745</v>
+        <v>1800</v>
       </c>
       <c r="N209" t="str">
         <v>N/A</v>
@@ -11428,7 +11428,7 @@
         <v>Critical</v>
       </c>
       <c r="M210">
-        <v>1780</v>
+        <v>1814</v>
       </c>
       <c r="N210" t="str">
         <v>N/A</v>
@@ -11479,7 +11479,7 @@
         <v>Critical</v>
       </c>
       <c r="M211">
-        <v>1777</v>
+        <v>1818</v>
       </c>
       <c r="N211" t="str">
         <v>N/A</v>
@@ -11530,7 +11530,7 @@
         <v>Critical</v>
       </c>
       <c r="M212">
-        <v>1801</v>
+        <v>1854</v>
       </c>
       <c r="N212" t="str">
         <v>N/A</v>
@@ -11581,7 +11581,7 @@
         <v>Critical</v>
       </c>
       <c r="M213">
-        <v>1803</v>
+        <v>1815</v>
       </c>
       <c r="N213" t="str">
         <v>N/A</v>
@@ -11632,7 +11632,7 @@
         <v>Critical</v>
       </c>
       <c r="M214">
-        <v>1787</v>
+        <v>1774</v>
       </c>
       <c r="N214" t="str">
         <v>N/A</v>
@@ -11683,7 +11683,7 @@
         <v>Critical</v>
       </c>
       <c r="M215">
-        <v>1833</v>
+        <v>1780</v>
       </c>
       <c r="N215" t="str">
         <v>N/A</v>
@@ -11734,7 +11734,7 @@
         <v>Critical</v>
       </c>
       <c r="M216">
-        <v>1864</v>
+        <v>1770</v>
       </c>
       <c r="N216" t="str">
         <v>N/A</v>
@@ -16466,7 +16466,7 @@
         <v>Critical</v>
       </c>
       <c r="M307">
-        <v>2068</v>
+        <v>2118</v>
       </c>
       <c r="N307" t="str">
         <v>N/A</v>
@@ -16518,7 +16518,7 @@
         <v>Critical</v>
       </c>
       <c r="M308">
-        <v>2097</v>
+        <v>2047</v>
       </c>
       <c r="N308" t="str">
         <v>N/A</v>
@@ -16570,7 +16570,7 @@
         <v>Critical</v>
       </c>
       <c r="M309">
-        <v>2069</v>
+        <v>2043</v>
       </c>
       <c r="N309" t="str">
         <v>N/A</v>
@@ -16622,7 +16622,7 @@
         <v>Critical</v>
       </c>
       <c r="M310">
-        <v>2188</v>
+        <v>2097</v>
       </c>
       <c r="N310" t="str">
         <v>N/A</v>
@@ -16674,7 +16674,7 @@
         <v>Critical</v>
       </c>
       <c r="M311">
-        <v>2222</v>
+        <v>2006</v>
       </c>
       <c r="N311" t="str">
         <v>N/A</v>
@@ -16726,7 +16726,7 @@
         <v>Critical</v>
       </c>
       <c r="M312">
-        <v>2418</v>
+        <v>2011</v>
       </c>
       <c r="N312" t="str">
         <v>N/A</v>
@@ -16778,7 +16778,7 @@
         <v>Critical</v>
       </c>
       <c r="M313">
-        <v>2198</v>
+        <v>2032</v>
       </c>
       <c r="N313" t="str">
         <v>N/A</v>
@@ -16830,7 +16830,7 @@
         <v>Critical</v>
       </c>
       <c r="M314">
-        <v>2231</v>
+        <v>2012</v>
       </c>
       <c r="N314" t="str">
         <v>N/A</v>
@@ -16882,7 +16882,7 @@
         <v>Critical</v>
       </c>
       <c r="M315">
-        <v>2101</v>
+        <v>2022</v>
       </c>
       <c r="N315" t="str">
         <v>N/A</v>
@@ -16934,7 +16934,7 @@
         <v>Critical</v>
       </c>
       <c r="M316">
-        <v>2089</v>
+        <v>1996</v>
       </c>
       <c r="N316" t="str">
         <v>N/A</v>
@@ -16986,7 +16986,7 @@
         <v>Critical</v>
       </c>
       <c r="M317">
-        <v>2081</v>
+        <v>2006</v>
       </c>
       <c r="N317" t="str">
         <v>N/A</v>
@@ -17038,7 +17038,7 @@
         <v>Critical</v>
       </c>
       <c r="M318">
-        <v>2070</v>
+        <v>1979</v>
       </c>
       <c r="N318" t="str">
         <v>N/A</v>
@@ -17090,7 +17090,7 @@
         <v>Critical</v>
       </c>
       <c r="M319">
-        <v>2090</v>
+        <v>2008</v>
       </c>
       <c r="N319" t="str">
         <v>N/A</v>
@@ -17142,7 +17142,7 @@
         <v>Critical</v>
       </c>
       <c r="M320">
-        <v>2038</v>
+        <v>2072</v>
       </c>
       <c r="N320" t="str">
         <v>N/A</v>
@@ -17194,7 +17194,7 @@
         <v>Critical</v>
       </c>
       <c r="M321">
-        <v>2032</v>
+        <v>2041</v>
       </c>
       <c r="N321" t="str">
         <v>N/A</v>
@@ -17246,7 +17246,7 @@
         <v>Critical</v>
       </c>
       <c r="M322">
-        <v>1972</v>
+        <v>2061</v>
       </c>
       <c r="N322" t="str">
         <v>N/A</v>
@@ -17298,7 +17298,7 @@
         <v>Critical</v>
       </c>
       <c r="M323">
-        <v>1996</v>
+        <v>2037</v>
       </c>
       <c r="N323" t="str">
         <v>N/A</v>
@@ -17350,7 +17350,7 @@
         <v>Critical</v>
       </c>
       <c r="M324">
-        <v>1934</v>
+        <v>2037</v>
       </c>
       <c r="N324" t="str">
         <v>N/A</v>
@@ -17402,7 +17402,7 @@
         <v>Critical</v>
       </c>
       <c r="M325">
-        <v>1995</v>
+        <v>2009</v>
       </c>
       <c r="N325" t="str">
         <v>N/A</v>
@@ -17454,7 +17454,7 @@
         <v>Critical</v>
       </c>
       <c r="M326">
-        <v>1990</v>
+        <v>2135</v>
       </c>
       <c r="N326" t="str">
         <v>N/A</v>

</xml_diff>